<commit_message>
Drop the README sheet from the sample VDDs
</commit_message>
<xml_diff>
--- a/sample_documents/DICT_Medicare Expansion-MIDS - Socially Determined.xlsx
+++ b/sample_documents/DICT_Medicare Expansion-MIDS - Socially Determined.xlsx
@@ -7,11 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FILES" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="demographics_package" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="analytics_package" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sd_ind_risk_data_package" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FILES" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="demographics_package" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="analytics_package" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sd_ind_risk_data_package" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -469,104 +468,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="110" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Vendor Data Dictionary — Socially Determined (SD), Michigan risk files</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr"/>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Purpose</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>The vendor-side input to the FRD-to-STTM agent. Together with the FRD (feed frame: files, tables, load strategy, DQ rules) and the client standards (target naming, typing, audit columns) it is sufficient to produce the STTM without reading any reference STTM.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>What it contains</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>FILES: one row per file the vendor delivers (pattern, format, delimiter, header row, cadence). One sheet per file: the fields in delivery order — name, vendor data type, length, whether the vendor guarantees a value, meaning, allowed values/range, an example value, PHI/PII.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>What it deliberately does NOT contain</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Anything the client decides: target schema/table/column names, stage/standard data types, mandatory-for-ETL flags, reject/recycle handling, audit columns (LOB, SRC_FILE_NAME, REC_CREATION_TIME, REC_UPDATED_TIME). Those come from the FRD and the standards documents.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>PROVENANCE — read this</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>This workbook was reverse-engineered on 2026-08-25 from the source-side band of the approved STTM (STTM_Medicare Expansion-MIDS - Socially Determined.xlsx) as a STAND-IN for the specification the vendor publishes. Field names, types, descriptions, ranges and examples are copied verbatim from that band. "Required" is derived from the STTM NULL CHECK column (NOT NULL -&gt; Y). Length is not stated anywhere in the STTM and is left blank. Replace this file with the vendor's real specification when it is obtained from the SharePoint project folder.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Known limitation</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>The two community files carry vendor type "String" on every field because that is what the STTM records; a real vendor spec would likely state numeric/percent types. Standard-layer promotion to Decimal(10,2)/Int is a client rule, not a vendor fact, and is out of scope here.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Legend</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Blue-shaded header rows are fixed. Every other cell is vendor-supplied fact. Y/N columns use exactly "Y" or "N".</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -781,7 +682,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4035,7 +3936,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -13970,7 +13871,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>